<commit_message>
fix: eval_pipeline and itext2kg max retries
</commit_message>
<xml_diff>
--- a/itext2kg_atom/datasets/atom/my_test_datasets/dataset_input_outzz.xlsx
+++ b/itext2kg_atom/datasets/atom/my_test_datasets/dataset_input_outzz.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['Chinese researchers stated that Chinese researchers identified a new virus.', 'The new virus is linked to an illness.', 'The illness has infected dozens of people across Asia.', 'The identification of the virus set off fears in a region.', 'The region was previously struck by a deadly epidemic on 2003-01-09.']</t>
+          <t>['Chinese researchers said Chinese researchers identified a new virus.', 'The new virus is behind an illness.', 'The illness has infected dozens of people across Asia.', 'The illness is setting off fears in a region.', 'The region was struck by a deadly epidemic on 2003-01-09.']</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['U.S. stock futures are down sharply.', 'The decline of U.S. stock futures occurred on 2020-01-27.', 'The decline of U.S. stock futures was caused by fears about the coronavirus outbreak.']</t>
+          <t>['U.S. stock futures are down sharply.', 'The decline in U.S. stock futures occurred on 2020-01-27.', 'Fears about the coronavirus outbreak caused U.S. stock futures to decline sharply.']</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>['President Trump’s lawyers open the third day of their defense on 2020-01-28.', 'An important question hangs over Washington regarding whether the Republican-controlled Senate will agree to hear testimony from witnesses.', 'The speaker flew to China at the beginning of January.', 'The speaker traveled to China to teach a three-week college class.', 'When the speaker flew to China at the beginning of January, the Wuhan coronavirus was barely on anyone’s radar.', 'By the time the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world.', 'On 2020-01-24, there were more than 800 cases of the Wuhan coronavirus in China.', 'By 2020-01-27, the total number of deaths from the Wuhan coronavirus was at least 80.', 'Apple is scheduled to report earnings on 2020-01-28.']</t>
+          <t>["President Trump's lawyers open the third day of their defense on 2020-01-28.", 'An important question hangs over Washington: Will the Republican-controlled Senate agree to hear testimony from witnesses?', 'The speaker flew to China at the beginning of January to teach a three-week college class.', 'When the speaker flew to China, the Wuhan coronavirus was barely on anyone’s radar.', 'By the time the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world.', 'By 2020-01-24, there were more than 800 cases of the Wuhan coronavirus in China.', 'By 2020-01-27, the total number of deaths from the Wuhan coronavirus was at least 80.', 'Apple is scheduled to report earnings on 2020-01-28.']</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['The World Health Organization declared a global health emergency on 2020-01-30.', 'The coronavirus outbreak spread well beyond China.', 'The coronavirus outbreak emerged in China during December 2019.']</t>
+          <t>['The World Health Organization declared a global health emergency on 2020-01-30.', 'The declaration by the World Health Organization occurred as the coronavirus outbreak spread well beyond China.', 'The coronavirus outbreak emerged in China.', 'The emergence of the coronavirus outbreak in China occurred in December 2019.']</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>['The whir of machines is echoing across a French factory floor in Angers, France, during the week of 2020-02-06.', 'The whir of machines is an unexpected result of the deadly virus.', 'The deadly virus nearly paralyzed cities in other parts of Asia.', 'Kolmi Hopen is the company.', 'Kolmi Hopen makes the medical face mask.', 'The medical face mask is suddenly one of the world’s hottest commodities.']</t>
+          <t>['The whir of machines is echoing across a French factory floor around 2020-02-06.', 'The echoing of machines is an unexpected result of the deadly virus.', 'The deadly virus nearly paralyzed cities in other parts of Asia.', 'Kolmi Hopen is the company.', 'Kolmi Hopen makes the medical face mask.', 'The medical face mask is suddenly one of the world’s hottest commodities.']</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>['The edition of Art Basel Hong Kong for 2020 was canceled.', 'Organizers cited the sudden and widespread outbreak of the coronavirus in China for the cancellation of Art Basel Hong Kong.', 'The Art Basel Hong Kong fair was held at the Hong Kong Convention and Exhibition Center.', 'The Art Basel Hong Kong fair was scheduled to run from March 17 through March 21.', 'Japan already had several confirmed coronavirus cases.', 'A giant cruise ship arrived at the port of Yokohama on 2020-01-27.', 'An alliance between Saudi Arabia and Russia helped prop up oil prices.', 'The support from the alliance between Saudi Arabia and Russia lasted for the last three years.', 'Saudi Arabia and Russia were not in perfect harmony on 2020-02-03.', 'Saudi Arabia and Russia tried to recalibrate production targets.', 'The recalibration of production targets was done to cope with reduced demand from China.', "China's economy was crippled by the coronavirus epidemic."]</t>
+          <t>["Art Basel Hong Kong's edition for on 2020-01-01 was canceled.", 'Organizers cited the sudden and widespread outbreak of the coronavirus in China as the reason for the cancellation.', 'The fair was scheduled to be held at the Hong Kong Convention and Exhibition Center.', 'The fair was scheduled to run from March 17 to March 21.', 'Japan already had several confirmed coronavirus cases.', 'A giant cruise ship arrived at the port of Yokohama on 2020-02-06.', 'An alliance between Saudi Arabia and Russia helped prop up oil prices.', 'The support from the alliance lasted for the last three years.', 'Saudi Arabia and Russia were not in perfect harmony on 2020-02-03.', 'Saudi Arabia and Russia tried to recalibrate production targets.', 'The recalibration was done to cope with reduced demand from China.', "China's economy has been crippled by the coronavirus epidemic."]</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09.', 'The death toll of the coronavirus epidemic in China exceeds the death toll of the SARS outbreak in 2003.', 'The development (the surpassing of the milestone) coincided with news.', 'World Health Organization experts might soon be in China.', 'World Health Organization experts might be in China to help stanch the crisis.']</t>
+          <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09.', 'The death toll of the coronavirus epidemic in China exceeds the death toll of the SARS outbreak on 2003-02-09.', 'The development (the high death toll) coincided with news.', 'World Health Organization experts might soon be in China.', 'The purpose of World Health Organization experts being in China is to help stanch the crisis.']</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>['Many people across China are returning to work on 2020-02-10.', 'The return to work followed an extended Lunar New Year break.', 'China is confronting two bleak statistics.']</t>
+          <t>['Many people across China are returning to work on 2020-02-10.', 'The Lunar New Year break was extended.', 'China is confronting two bleak statistics.']</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>['The family from Shanghai was vacationing in Singapore.', 'The family from Shanghai learned that the new coronavirus arrived in Singapore from China.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways when making decisions involving risks.', 'The coronavirus epidemic has been known as the Asian disease problem.', 'Federal authorities said on 2020-02-10 that a woman sick from the coronavirus was released from a San Diego hospital.', 'The release of the woman was caused by a labeling error on samples to be tested for the virus.', 'The labeling error led officials to incorrectly indicate that the woman was not infected.', 'Chinese health officials said on 2020-02-10 that the death toll from the coronavirus had passed 1,000.']</t>
+          <t>['The family from Shanghai was vacationing in Singapore in January 2020.', 'The family from Shanghai learned that the new coronavirus arrived in Singapore from China.', 'Humans can be irrational in systematic ways when making decisions that involve risks.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways.', 'Amos Tversky and Daniel Kahneman used a hypothetical situation to demonstrate the fact.', 'The coronavirus epidemic has come to be known as the Asian disease problem.', 'A woman sick from the coronavirus was released from a San Diego hospital on 2020-02-10.', 'The release occurred after a labeling error on samples tested for the virus.', 'The labeling error led officials to incorrectly indicate that the woman was not infected.', 'Federal authorities stated this on 2020-02-10.', 'Chinese health officials stated on 2020-02-10 that the death toll from the coronavirus had passed 1,000.']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: massive bugfix (see description)
+ disabled LLM models thinking/reasoning: lantency and numbers of quintuples extracted increased
+ fixed bad embeddings computation by replacing '_' with ' ' in entities and relationships. Also migrated from nomic-embed-text to qwen2-1.5b-instruct model.
+ edit start-llama-servers: pooling last for qwen
</commit_message>
<xml_diff>
--- a/itext2kg_atom/datasets/atom/my_test_datasets/dataset_input_outzz.xlsx
+++ b/itext2kg_atom/datasets/atom/my_test_datasets/dataset_input_outzz.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>['Chinese researchers said Chinese researchers identified a new virus.', 'The new virus is behind an illness.', 'The illness has infected dozens of people across Asia.', 'The illness is setting off fears in a region.', 'The region was struck by a deadly epidemic on 2003-01-09.']</t>
+          <t>['Chinese researchers identified a new virus.', 'The new virus is behind an illness that has infected dozens of people across Asia.', 'The illness has infected dozens of people across Asia.', 'The region was struck by a deadly epidemic on 2003-01-09 2020-01-09.']</t>
         </is>
       </c>
     </row>
@@ -519,7 +519,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>['The spread of a mysterious respiratory virus prompted the authorities to limit travel.', 'The authorities limited travel in cities in China.', 'Wuhan is a city in China.', 'The mysterious respiratory virus was first found in Wuhan in December 2019.', 'The mysterious respiratory virus spread across China.', 'The mysterious respiratory virus spread to at least 10 other countries.']</t>
+          <t>['Authorities have limited travel in cities in China.', 'Wuhan is one of the cities where authorities limited travel.', 'The mysterious respiratory virus was first found in Wuhan in December 2019.', 'The mysterious respiratory virus has spread across China.', 'The mysterious respiratory virus has spread to at least 10 other countries.']</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>['U.S. stock futures are down sharply.', 'The decline in U.S. stock futures occurred on 2020-01-27.', 'Fears about the coronavirus outbreak caused U.S. stock futures to decline sharply.']</t>
+          <t>['On 2020-01-27, U.S. stock futures were down sharply.', 'The sharp decline in U.S. stock futures on 2020-01-27 was caused by fears about the coronavirus outbreak.']</t>
         </is>
       </c>
     </row>
@@ -585,7 +585,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>["President Trump's lawyers open the third day of their defense on 2020-01-28.", 'An important question hangs over Washington: Will the Republican-controlled Senate agree to hear testimony from witnesses?', 'The speaker flew to China at the beginning of January to teach a three-week college class.', 'When the speaker flew to China, the Wuhan coronavirus was barely on anyone’s radar.', 'By the time the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world.', 'By 2020-01-24, there were more than 800 cases of the Wuhan coronavirus in China.', 'By 2020-01-27, the total number of deaths from the Wuhan coronavirus was at least 80.', 'Apple is scheduled to report earnings on 2020-01-28.']</t>
+          <t>['On 2020-01-27, President Trump’s lawyers opened the third day of their defense.', 'On 2020-01-27, a question existed regarding whether the Republican-controlled Senate would agree to hear testimony from witnesses.', 'The author flew to China at the beginning of January 2020 to teach a three-week college class.', 'The Wuhan coronavirus was barely on anyone’s radar at the beginning of January 2020.', 'The author returned to New York on 2020-01-24.', 'By 2020-01-24, the Wuhan coronavirus was front page news around the world.', 'By 2020-01-24, there were more than 800 cases of the Wuhan coronavirus in China.', 'By 2020-01-27, the total number of deaths from the Wuhan coronavirus was at least 80.', 'Apple is scheduled to report earnings on 2020-01-27.']</t>
         </is>
       </c>
     </row>
@@ -618,7 +618,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>['The World Health Organization declared a global health emergency on 2020-01-30.', 'The declaration by the World Health Organization occurred as the coronavirus outbreak spread well beyond China.', 'The coronavirus outbreak emerged in China.', 'The emergence of the coronavirus outbreak in China occurred in December 2019.']</t>
+          <t>['The World Health Organization declared a global health emergency on 2020-01-29.', 'The coronavirus outbreak spread well beyond China.', 'The coronavirus outbreak emerged in China in December 2019.']</t>
         </is>
       </c>
     </row>
@@ -651,7 +651,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>['The whir of machines is echoing across a French factory floor around 2020-02-06.', 'The echoing of machines is an unexpected result of the deadly virus.', 'The deadly virus nearly paralyzed cities in other parts of Asia.', 'Kolmi Hopen is the company.', 'Kolmi Hopen makes the medical face mask.', 'The medical face mask is suddenly one of the world’s hottest commodities.']</t>
+          <t>['On 2020-02-06, machines were operating in a factory in Angers, France.', 'The factory is located in Angers, France.', 'The company is named Kolmi Hopen.', 'Kolmi Hopen produces medical face masks.', "Medical face masks became one of the world's hottest commodities.", 'A deadly virus nearly paralyzed cities in other parts of Asia.', 'The production of medical face masks by Kolmi Hopen is a result of the deadly virus.']</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>["Art Basel Hong Kong's edition for on 2020-01-01 was canceled.", 'Organizers cited the sudden and widespread outbreak of the coronavirus in China as the reason for the cancellation.', 'The fair was scheduled to be held at the Hong Kong Convention and Exhibition Center.', 'The fair was scheduled to run from March 17 to March 21.', 'Japan already had several confirmed coronavirus cases.', 'A giant cruise ship arrived at the port of Yokohama on 2020-02-06.', 'An alliance between Saudi Arabia and Russia helped prop up oil prices.', 'The support from the alliance lasted for the last three years.', 'Saudi Arabia and Russia were not in perfect harmony on 2020-02-03.', 'Saudi Arabia and Russia tried to recalibrate production targets.', 'The recalibration was done to cope with reduced demand from China.', "China's economy has been crippled by the coronavirus epidemic."]</t>
+          <t>['Art Basel Hong Kong was canceled for the 2020 edition.', 'Organizers cited the sudden and widespread outbreak of the coronavirus in China as the reason for the cancellation of Art Basel Hong Kong.', 'Art Basel Hong Kong was scheduled to run from 2020-03-17 through 2020-03-21.', 'Art Basel Hong Kong was to be held at the Hong Kong Convention and Exhibition Center.', 'Art Basel Hong Kong was to feature premier galleries from Asia and beyond.', 'Japan had several confirmed coronavirus cases by 2020-02-07.', 'A giant cruise ship arrived at the port of Yokohama on 2020-01-30.', 'An alliance between Saudi Arabia and Russia helped prop up oil prices for the three years preceding 2020-02-07.', 'Saudi Arabia and Russia were not in perfect harmony during the week of 2020-02-03.', 'Saudi Arabia and Russia tried to recalibrate production targets during the week of 2020-02-03.', 'Saudi Arabia and Russia tried to recalibrate production targets to cope with reduced demand from China.', 'The economy of China was crippled by the coronavirus epidemic.', 'The coronavirus epidemic caused reduced demand from China.']</t>
         </is>
       </c>
     </row>
@@ -717,7 +717,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09.', 'The death toll of the coronavirus epidemic in China exceeds the death toll of the SARS outbreak on 2003-02-09.', 'The development (the high death toll) coincided with news.', 'World Health Organization experts might soon be in China.', 'The purpose of World Health Organization experts being in China is to help stanch the crisis.']</t>
+          <t>['On 2020-02-08, the coronavirus death toll in China exceeded the death toll of the SARS outbreak from 17 years prior.', 'On 2020-02-08, news emerged that World Health Organization experts might soon enter China.', "The purpose of the World Health Organization experts' visit is to help stanch the coronavirus crisis."]</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>['Many people across China are returning to work on 2020-02-10.', 'The Lunar New Year break was extended.', 'China is confronting two bleak statistics.']</t>
+          <t>['On 2020-02-10, many people across China returned to work.', 'The Lunar New Year break was already extended before 2020-02-10.', 'China is confronting two bleak statistics on 2020-02-10.']</t>
         </is>
       </c>
     </row>
@@ -783,7 +783,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>['The family from Shanghai was vacationing in Singapore in January 2020.', 'The family from Shanghai learned that the new coronavirus arrived in Singapore from China.', 'Humans can be irrational in systematic ways when making decisions that involve risks.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways.', 'Amos Tversky and Daniel Kahneman used a hypothetical situation to demonstrate the fact.', 'The coronavirus epidemic has come to be known as the Asian disease problem.', 'A woman sick from the coronavirus was released from a San Diego hospital on 2020-02-10.', 'The release occurred after a labeling error on samples tested for the virus.', 'The labeling error led officials to incorrectly indicate that the woman was not infected.', 'Federal authorities stated this on 2020-02-10.', 'Chinese health officials stated on 2020-02-10 that the death toll from the coronavirus had passed 1,000.']</t>
+          <t>['A family from Shanghai was vacationing in Singapore in January 2020.', 'The family from Shanghai learned that the new coronavirus had arrived in Singapore in January 2020.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways when making decisions involving risks.', 'The Asian disease problem is a hypothetical situation used by Amos Tversky and Daniel Kahneman to demonstrate human irrationality.', 'A woman sick from the coronavirus was released from a San Diego hospital during the week of 2020-02-03.', 'A labeling error on samples to be tested for the virus led officials to incorrectly indicate that a woman was not infected.', 'Federal authorities announced the release of the woman from the San Diego hospital on 2020-02-10.', 'Chinese health officials reported that the death toll from the coronavirus passed 1,000 on 2020-02-10.', 'The text provides updates and maps of where the coronavirus has reached as of 2020-02-10.']</t>
         </is>
       </c>
     </row>

</xml_diff>